<commit_message>
[21 10] add excel_pivot.py
</commit_message>
<xml_diff>
--- a/day_21_6_09_2025/tabela_przestawna.xlsx
+++ b/day_21_6_09_2025/tabela_przestawna.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dane" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabela Przestawna" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabele Przestawna" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -435,7 +435,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Sprzedaż</t>
+          <t>Sprzedaj</t>
         </is>
       </c>
     </row>
@@ -536,7 +536,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>3200</v>
+        <v>1500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>